<commit_message>
Fix special assay Excel footer and template alignment
</commit_message>
<xml_diff>
--- a/app/templates/Template_Azul_Metileno.xlsx
+++ b/app/templates/Template_Azul_Metileno.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2C00AEDE-D2A5-4F1F-82CC-4A2D8F02A3B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{154F03C7-D398-4D1C-AE82-E56E82BA1521}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -176,7 +176,7 @@
     <numFmt numFmtId="165" formatCode="0\ &quot;/ CO-06&quot;"/>
     <numFmt numFmtId="166" formatCode="&quot;FORMATO F-LEM-P-SU-11.01&quot;"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -258,19 +258,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="8"/>
-      <color theme="0"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="8"/>
-      <color theme="0"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
@@ -679,52 +666,52 @@
       <alignment vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="10" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -741,10 +728,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
@@ -809,10 +792,6 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="1" fontId="14" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -822,18 +801,6 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="20" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="18" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="20" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -851,14 +818,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="13" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -877,6 +836,34 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -1828,30 +1815,30 @@
       <c r="I6" s="48"/>
     </row>
     <row r="7" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="72" t="s">
+      <c r="A7" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="72"/>
-      <c r="C7" s="72"/>
-      <c r="D7" s="72"/>
-      <c r="E7" s="72"/>
-      <c r="F7" s="72"/>
-      <c r="G7" s="72"/>
-      <c r="H7" s="72"/>
-      <c r="I7" s="72"/>
+      <c r="B7" s="71"/>
+      <c r="C7" s="71"/>
+      <c r="D7" s="71"/>
+      <c r="E7" s="71"/>
+      <c r="F7" s="71"/>
+      <c r="G7" s="71"/>
+      <c r="H7" s="71"/>
+      <c r="I7" s="71"/>
     </row>
     <row r="8" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="73" t="s">
+      <c r="A8" s="72" t="s">
         <v>37</v>
       </c>
-      <c r="B8" s="73"/>
-      <c r="C8" s="73"/>
-      <c r="D8" s="73"/>
-      <c r="E8" s="73"/>
-      <c r="F8" s="73"/>
-      <c r="G8" s="73"/>
-      <c r="H8" s="73"/>
-      <c r="I8" s="73"/>
+      <c r="B8" s="72"/>
+      <c r="C8" s="72"/>
+      <c r="D8" s="72"/>
+      <c r="E8" s="72"/>
+      <c r="F8" s="72"/>
+      <c r="G8" s="72"/>
+      <c r="H8" s="72"/>
+      <c r="I8" s="72"/>
       <c r="M8"/>
     </row>
     <row r="9" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
@@ -1866,20 +1853,20 @@
       <c r="I9" s="38"/>
     </row>
     <row r="10" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="97" t="s">
+      <c r="B10" s="90" t="s">
         <v>39</v>
       </c>
-      <c r="C10" s="98"/>
-      <c r="D10" s="96" t="s">
+      <c r="C10" s="91"/>
+      <c r="D10" s="89" t="s">
         <v>40</v>
       </c>
-      <c r="E10" s="96" t="s">
+      <c r="E10" s="89" t="s">
         <v>41</v>
       </c>
-      <c r="F10" s="97" t="s">
+      <c r="F10" s="90" t="s">
         <v>42</v>
       </c>
-      <c r="G10" s="98"/>
+      <c r="G10" s="91"/>
       <c r="H10"/>
       <c r="I10"/>
       <c r="J10" s="49"/>
@@ -1887,12 +1874,12 @@
     </row>
     <row r="11" spans="1:13" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="19"/>
-      <c r="B11" s="97"/>
-      <c r="C11" s="98"/>
-      <c r="D11" s="99"/>
-      <c r="E11" s="99"/>
-      <c r="F11" s="97"/>
-      <c r="G11" s="98"/>
+      <c r="B11" s="90"/>
+      <c r="C11" s="91"/>
+      <c r="D11" s="92"/>
+      <c r="E11" s="92"/>
+      <c r="F11" s="90"/>
+      <c r="G11" s="91"/>
       <c r="H11"/>
       <c r="I11"/>
       <c r="J11" s="49"/>
@@ -1912,32 +1899,32 @@
       <c r="K12" s="49"/>
     </row>
     <row r="13" spans="1:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="74" t="s">
+      <c r="A13" s="73" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="75"/>
-      <c r="C13" s="75"/>
-      <c r="D13" s="75"/>
-      <c r="E13" s="75"/>
-      <c r="F13" s="75"/>
-      <c r="G13" s="75"/>
-      <c r="H13" s="75"/>
-      <c r="I13" s="76"/>
+      <c r="B13" s="74"/>
+      <c r="C13" s="74"/>
+      <c r="D13" s="74"/>
+      <c r="E13" s="74"/>
+      <c r="F13" s="74"/>
+      <c r="G13" s="74"/>
+      <c r="H13" s="74"/>
+      <c r="I13" s="75"/>
       <c r="J13" s="49"/>
       <c r="K13" s="49"/>
     </row>
     <row r="14" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="69" t="s">
+      <c r="A14" s="68" t="s">
         <v>36</v>
       </c>
-      <c r="B14" s="70"/>
-      <c r="C14" s="70"/>
-      <c r="D14" s="70"/>
-      <c r="E14" s="70"/>
-      <c r="F14" s="70"/>
-      <c r="G14" s="70"/>
-      <c r="H14" s="70"/>
-      <c r="I14" s="71"/>
+      <c r="B14" s="69"/>
+      <c r="C14" s="69"/>
+      <c r="D14" s="69"/>
+      <c r="E14" s="69"/>
+      <c r="F14" s="69"/>
+      <c r="G14" s="69"/>
+      <c r="H14" s="69"/>
+      <c r="I14" s="70"/>
       <c r="J14" s="49"/>
       <c r="K14" s="49"/>
     </row>
@@ -1956,29 +1943,29 @@
     </row>
     <row r="16" spans="1:13" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="50"/>
-      <c r="B16" s="87" t="s">
+      <c r="B16" s="82" t="s">
         <v>31</v>
       </c>
-      <c r="C16" s="88"/>
-      <c r="D16" s="88"/>
+      <c r="C16" s="83"/>
+      <c r="D16" s="83"/>
       <c r="E16" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="F16" s="89" t="s">
+      <c r="F16" s="84" t="s">
         <v>18</v>
       </c>
-      <c r="G16" s="89"/>
+      <c r="G16" s="84"/>
       <c r="I16" s="51"/>
       <c r="J16" s="49"/>
       <c r="K16" s="52"/>
     </row>
     <row r="17" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="50"/>
-      <c r="B17" s="90" t="s">
+      <c r="B17" s="85" t="s">
         <v>20</v>
       </c>
-      <c r="C17" s="91"/>
-      <c r="D17" s="92"/>
+      <c r="C17" s="86"/>
+      <c r="D17" s="87"/>
       <c r="E17" s="30" t="s">
         <v>21</v>
       </c>
@@ -2000,10 +1987,10 @@
       <c r="E18" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="F18" s="63">
+      <c r="F18" s="95">
         <v>10</v>
       </c>
-      <c r="G18" s="63"/>
+      <c r="G18" s="95"/>
       <c r="I18" s="51"/>
       <c r="J18" s="53"/>
       <c r="K18" s="52"/>
@@ -2018,8 +2005,8 @@
       <c r="E19" s="31" t="s">
         <v>24</v>
       </c>
-      <c r="F19" s="85"/>
-      <c r="G19" s="86"/>
+      <c r="F19" s="96"/>
+      <c r="G19" s="97"/>
       <c r="I19" s="51"/>
       <c r="J19" s="53"/>
       <c r="K19" s="52"/>
@@ -2034,29 +2021,29 @@
       <c r="E20" s="31" t="s">
         <v>24</v>
       </c>
-      <c r="F20" s="80">
+      <c r="F20" s="98">
         <v>10</v>
       </c>
-      <c r="G20" s="80"/>
+      <c r="G20" s="98"/>
       <c r="I20" s="51"/>
       <c r="J20" s="49"/>
       <c r="K20" s="49"/>
     </row>
     <row r="21" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="50"/>
-      <c r="B21" s="81" t="s">
+      <c r="B21" s="79" t="s">
         <v>25</v>
       </c>
-      <c r="C21" s="82"/>
-      <c r="D21" s="83"/>
+      <c r="C21" s="80"/>
+      <c r="D21" s="81"/>
       <c r="E21" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="F21" s="84">
+      <c r="F21" s="99">
         <f>F17*F18/F20</f>
         <v>5</v>
       </c>
-      <c r="G21" s="84"/>
+      <c r="G21" s="99"/>
       <c r="I21" s="51"/>
       <c r="J21" s="49"/>
       <c r="K21" s="49"/>
@@ -2111,26 +2098,26 @@
       <c r="K27" s="49"/>
     </row>
     <row r="28" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E28" s="77" t="s">
+      <c r="E28" s="76" t="s">
         <v>28</v>
       </c>
-      <c r="F28" s="79"/>
-      <c r="G28" s="77" t="s">
+      <c r="F28" s="78"/>
+      <c r="G28" s="76" t="s">
         <v>29</v>
       </c>
-      <c r="H28" s="78"/>
-      <c r="I28" s="79"/>
+      <c r="H28" s="77"/>
+      <c r="I28" s="78"/>
       <c r="J28" s="49"/>
       <c r="K28" s="49"/>
     </row>
     <row r="29" spans="1:11" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E29" s="64" t="s">
+      <c r="E29" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="F29" s="65"/>
-      <c r="G29" s="66"/>
-      <c r="H29" s="67"/>
-      <c r="I29" s="68"/>
+      <c r="F29" s="64"/>
+      <c r="G29" s="65"/>
+      <c r="H29" s="66"/>
+      <c r="I29" s="67"/>
       <c r="J29" s="49"/>
       <c r="K29" s="49"/>
     </row>
@@ -2139,13 +2126,13 @@
       <c r="B30" s="41"/>
       <c r="C30" s="41"/>
       <c r="D30" s="41"/>
-      <c r="E30" s="64" t="s">
+      <c r="E30" s="63" t="s">
         <v>30</v>
       </c>
-      <c r="F30" s="65"/>
-      <c r="G30" s="66"/>
-      <c r="H30" s="67"/>
-      <c r="I30" s="68"/>
+      <c r="F30" s="64"/>
+      <c r="G30" s="65"/>
+      <c r="H30" s="66"/>
+      <c r="I30" s="67"/>
       <c r="J30" s="49"/>
       <c r="K30" s="49"/>
     </row>
@@ -2397,10 +2384,10 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="95" t="s">
+      <c r="A2" s="88" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="95"/>
+      <c r="B2" s="88"/>
       <c r="C2" s="5" t="s">
         <v>10</v>
       </c>

</xml_diff>